<commit_message>
loading script for ploting RvsSBML validation results
</commit_message>
<xml_diff>
--- a/Input/Parameters.GSA.xlsx
+++ b/Input/Parameters.GSA.xlsx
@@ -3115,8 +3115,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002AA8BEAC825CAE4DA772B4C276EF423C" ma:contentTypeVersion="12" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="d181a0c76d3b9cd5602d3d2c9a9fc37e">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="568ff3df-f16a-482d-bb3c-58af1efa1658" xmlns:ns3="13cea704-446d-46be-be94-9e10425fef80" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f04bd294d33ae414712fbbf90740e85a" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002AA8BEAC825CAE4DA772B4C276EF423C" ma:contentTypeVersion="12" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="08e2132e63c6ee1d6b0a0758f6c0554f">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="568ff3df-f16a-482d-bb3c-58af1efa1658" xmlns:ns3="13cea704-446d-46be-be94-9e10425fef80" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0ed1ebf33a67d32129b0ef2e0882217b" ns2:_="" ns3:_="">
     <xsd:import namespace="568ff3df-f16a-482d-bb3c-58af1efa1658"/>
     <xsd:import namespace="13cea704-446d-46be-be94-9e10425fef80"/>
     <xsd:element name="properties">
@@ -3345,7 +3345,7 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B7892EC9-8941-4732-9E22-55170B655489}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED1E687C-9DB1-4722-8D88-EAA6C91461CA}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>